<commit_message>
updated MTS and added MTS section to race video analysis
</commit_message>
<xml_diff>
--- a/pages/video_analysis/MTS_Master_Men.xlsx
+++ b/pages/video_analysis/MTS_Master_Men.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G57"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -898,10 +898,486 @@
         <v/>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B30">
+        <v>12.48</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Rider 3 Forward</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Jaxson Russell</v>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B31">
+        <v>12.48</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Rider 2 Forward</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Luke Blackwood</v>
+      </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B32">
+        <v>12.5</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Start</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Alex Schuler</v>
+      </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B33">
+        <v>12.52</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Rider 1 Forward</v>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B34">
+        <v>19.482</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B35">
+        <v>19.85</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B36">
+        <v>20.05</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B37">
+        <v>23.467</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B38">
+        <v>23.792</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B39">
+        <v>23.952</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B40">
+        <v>26.952</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B41">
+        <v>27.204</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B42">
+        <v>27.344</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B43">
+        <v>30.324</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B44">
+        <v>30.464</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B45">
+        <v>30.584</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B46">
+        <v>33.664</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B47">
+        <v>33.804</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B48">
+        <v>36.864</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B49">
+        <v>36.964</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B50">
+        <v>40.124</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B51">
+        <v>40.244</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B52">
+        <v>43.484</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B53">
+        <v>43.544</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B54">
+        <v>46.844</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B55">
+        <v>50.084</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B56">
+        <v>53.404</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>26-02-10 Oceania's CCh Devo1 Q</v>
+      </c>
+      <c r="B57">
+        <v>56.764</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Marker</v>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G57"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>